<commit_message>
fix: prove provider credential lifecycle
</commit_message>
<xml_diff>
--- a/docs/feature-status/hermes-feature-status.xlsx
+++ b/docs/feature-status/hermes-feature-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf6aef3a726124f86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Status" sheetId="2" r:id="R3e4da1c4d3034d8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Index" sheetId="3" r:id="Rd1ae8c78340b47ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Log" sheetId="4" r:id="Rf5e0e850309343f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R70510b7262d744a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Status" sheetId="2" r:id="R376e2a08d8b74cfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Index" sheetId="3" r:id="R06f8150ef2434597"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Log" sheetId="4" r:id="R9844f66d87d341d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -172,7 +172,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ValidationLogTable" displayName="ValidationLogTable" ref="A1:D52" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ValidationLogTable" displayName="ValidationLogTable" ref="A1:D56" headerRowCount="1">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="When"/>
     <x:tableColumn id="2" name="Command"/>
@@ -813,7 +813,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bc8ceb080e9463e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e028655c3af4352"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1038,13 +1038,13 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="H5" s="13" t="str">
-        <x:v>PASS: App/provider install-gate tests; manual credential QA pending</x:v>
+        <x:v>PASS: App/provider install-gate tests plus provider-flow smoke; no plaintext key leak observed</x:v>
       </x:c>
       <x:c r="I5" s="13" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="J5" s="9" t="str">
-        <x:v>Launch with no key, save provider key, verify onboarding/workspace transition and key redaction.</x:v>
+        <x:v>Launch throwaway installed home with no key; verify Setup gate, save/update/remove OpenRouter, relaunch to no-key gate, and confirm .env/log redaction.</x:v>
       </x:c>
       <x:c r="K5" s="9" t="str">
         <x:v>2026-06-22</x:v>
@@ -1054,7 +1054,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="N5" s="9" t="str">
-        <x:v>npx vitest run src/renderer/src/App.test.tsx tests/install-gate-providers.test.ts tests/providers.test.ts: passed in focused slices.</x:v>
+        <x:v>npx vitest run tests/keychain-env.test.ts tests/credential-pool-schema.test.ts tests/hermes-auth.test.ts tests/validation.test.ts src/renderer/src/screens/Providers/Providers.test.tsx tests/install-gate-providers.test.ts tests/providers.test.ts tests/preload-api-surface.test.ts; node scripts/provider-flow-smoke.mjs: PROVIDER_FLOW_SMOKE_OK (no-key gate, setup save, update/remove, relaunch).</x:v>
       </x:c>
       <x:c r="O5" s="9" t="str"/>
     </x:row>
@@ -1306,13 +1306,13 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="H11" s="13" t="str">
-        <x:v>PASS: Providers.test.tsx and provider backend tests; manual credential QA pending</x:v>
+        <x:v>PASS: Providers.test.tsx, provider backend tests, and provider-flow smoke; live OAuth account QA remains opt-in</x:v>
       </x:c>
       <x:c r="I11" s="13" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="J11" s="9" t="str">
-        <x:v>Add/remove/test API-key provider, sign in/out OAuth provider, inspect update routine controls.</x:v>
+        <x:v>Add/update/remove API-key provider; deterministic Nous OAuth sign-in/out via modal/IPC; optional live OAuth browser/account pass with scripts/drive-nous-oauth.js.</x:v>
       </x:c>
       <x:c r="K11" s="9" t="str">
         <x:v>2026-06-22</x:v>
@@ -1322,7 +1322,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="N11" s="9" t="str">
-        <x:v>npx vitest run src/renderer/src/screens/Providers/Providers.test.tsx plus provider/model backend tests: passed in focused slices.</x:v>
+        <x:v>npx vitest run tests/keychain-env.test.ts tests/credential-pool-schema.test.ts tests/hermes-auth.test.ts tests/validation.test.ts src/renderer/src/screens/Providers/Providers.test.tsx tests/install-gate-providers.test.ts tests/providers.test.ts tests/preload-api-surface.test.ts; node scripts/provider-flow-smoke.mjs: PROVIDER_FLOW_SMOKE_OK (provider lifecycle plus deterministic Nous OAuth).</x:v>
       </x:c>
       <x:c r="O11" s="9" t="str"/>
     </x:row>
@@ -4297,7 +4297,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R279e99a491554a75"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32ecfe1521c7402b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4425,7 +4425,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R137f6bd2bb12448f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc466a58d4af349d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5168,10 +5168,66 @@
         <x:v>14/14 behavior screenshots passed after adding Journal coverage: create entry, edit title/body, return to timeline, set mood, reopen entry, and verify journal markdown frontmatter/body.</x:v>
       </x:c>
     </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>2026-06-22</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>npx vitest run tests/keychain-env.test.ts tests/credential-pool-schema.test.ts tests/hermes-auth.test.ts tests/validation.test.ts src/renderer/src/screens/Providers/Providers.test.tsx tests/install-gate-providers.test.ts tests/providers.test.ts tests/preload-api-surface.test.ts</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>8 files passed; 254 tests passed. Covers keychain blank removal, provider UI removal, credential pool/OAuth/auth validation, install gate, provider registry, and preload parity.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>2026-06-22</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>npm run typecheck</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D54" t="str">
+        <x:v>typecheck:node and typecheck:web completed successfully.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
+        <x:v>2026-06-22</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>npm run build</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D55" t="str">
+        <x:v>OCR assets ready, typecheck passed, MCP bundles built, and Electron/Vite build completed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="str">
+        <x:v>2026-06-22</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>node scripts/provider-flow-smoke.mjs</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D56" t="str">
+        <x:v>PROVIDER_FLOW_SMOKE_OK; proved no-key startup gate, Setup save, provider update/remove, relaunch no-key gate, deterministic Nous OAuth sign-in/out, and no plaintext key in .env/app logs.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7df35612f27743ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd813bdd24ced42ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
test: cover fresh personal health flow
</commit_message>
<xml_diff>
--- a/docs/feature-status/hermes-feature-status.xlsx
+++ b/docs/feature-status/hermes-feature-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R70510b7262d744a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Status" sheetId="2" r:id="R376e2a08d8b74cfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Index" sheetId="3" r:id="R06f8150ef2434597"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Log" sheetId="4" r:id="R9844f66d87d341d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R194047822de344ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Status" sheetId="2" r:id="R970f07da0277465b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Index" sheetId="3" r:id="R8d336a2ff9fa40b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Log" sheetId="4" r:id="R50ab5db673d9429a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -813,7 +813,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e028655c3af4352"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re070846d35084118"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3913,7 +3913,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="H70" s="13" t="str">
-        <x:v>PASS: sps-surfaces-smoke; profile/delete/digest manual QA pending</x:v>
+        <x:v>PASS: sps-surfaces-smoke covers fresh/offline profile, journal/protocol/doc delete paths, and offline clinical digest.</x:v>
       </x:c>
       <x:c r="I70" s="13" t="str">
         <x:v>P1</x:v>
@@ -3931,9 +3931,11 @@
         <x:v>Fixed</x:v>
       </x:c>
       <x:c r="N70" s="9" t="str">
-        <x:v>npx vitest run tests/db-pool.test.ts: 7 tests passed, including missing writable DB creation and metadata trigger skip when messages is absent. npm run build passed. DEBUG=pw:browser* node scripts/sps-surfaces-smoke.mjs: health journal/biometrics, peptide protocol creation, Medical Vault simulated scan, and no metadata-trigger error.</x:v>
-      </x:c>
-      <x:c r="O70" s="9" t="str"/>
+        <x:v>npx vitest run tests/db-pool.test.ts src/renderer/src/screens/SpsAgent/store/workspace-dbcleanup.test.ts: 11 tests passed. npm run build passed. DEBUG=pw:browser* node scripts/sps-surfaces-smoke.mjs: 15/15 behavior screenshots passed; HEALTH_DELETE_OK journal entry, medication protocol, and medical document; HEALTH_DIGEST_OK 2 offline clinical articles; no targeted health bootstrap console/page errors.</x:v>
+      </x:c>
+      <x:c r="O70" s="9" t="str">
+        <x:v>Delete and digest proof is now covered in the fresh/offline smoke; broader live clinical RSS source UX remains outside this HF-069 gate.</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="9" t="str">
@@ -4297,7 +4299,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32ecfe1521c7402b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94205b57b63c4b21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4425,7 +4427,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc466a58d4af349d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raff9ad353b18497f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5224,10 +5226,24 @@
         <x:v>PROVIDER_FLOW_SMOKE_OK; proved no-key startup gate, Setup save, provider update/remove, relaunch no-key gate, deterministic Nous OAuth sign-in/out, and no plaintext key in .env/app logs.</x:v>
       </x:c>
     </x:row>
+    <x:row r="57">
+      <x:c r="A57" t="str">
+        <x:v>2026-06-22</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>DEBUG=pw:browser* node scripts/sps-surfaces-smoke.mjs</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D57" t="str">
+        <x:v>15/15 behavior screenshots passed. Personal Health fresh/offline checks covered journal/protocol/document deletes via UI plus IPC readback, offline clinical digest render with 2 fallback articles, and no targeted health bootstrap console/page errors.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd813bdd24ced42ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b702bd8f58b4e18"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix SPS page-tree trash restore
</commit_message>
<xml_diff>
--- a/docs/feature-status/hermes-feature-status.xlsx
+++ b/docs/feature-status/hermes-feature-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R194047822de344ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Status" sheetId="2" r:id="R970f07da0277465b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Index" sheetId="3" r:id="R8d336a2ff9fa40b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Log" sheetId="4" r:id="R50ab5db673d9429a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re1dfc1fd9c4b4f67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Status" sheetId="2" r:id="R23b8f8992c4549d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Index" sheetId="3" r:id="R419d13529f6048f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Log" sheetId="4" r:id="Rc04dee35db7e45a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -813,7 +813,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re070846d35084118"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0212ab0474634df4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1873,7 +1873,7 @@
         <x:v>Implemented</x:v>
       </x:c>
       <x:c r="H24" s="13" t="str">
-        <x:v>PASS: sidebar/tree-adjacent tests and sps-surfaces-smoke; manual DnD QA pending</x:v>
+        <x:v>PASS: nested restore/permanent-delete store tests, TreeNode drag/drop tests, storage cleanup tests, build, and sps-surfaces-smoke DnD/trash coverage</x:v>
       </x:c>
       <x:c r="I24" s="13" t="str">
         <x:v>P0</x:v>
@@ -1889,7 +1889,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="N24" s="9" t="str">
-        <x:v>Renderer slice included Sidebar and SidebarRecents tests. node scripts/sps-surfaces-smoke.mjs: page menu created a subpage, renamed it, moved it to trash, restored it, and the Trash row covered permanent delete. Drag/drop remains manual behavior QA.</x:v>
+        <x:v>npm test -- --run src/renderer/src/screens/SpsAgent/store/workspace-dbcleanup.test.ts src/renderer/src/screens/SpsAgent/lib/tree.test.ts src/renderer/src/screens/SpsAgent/sidebar/TreeNode.test.tsx: 3 files, 14 tests passed. npm test -- --run src/main/sps-vault.test.ts src/renderer/src/screens/SpsAgent/lib/vaultStore.test.ts: 2 files, 40 tests passed. npm run typecheck: node+web passed. npm run build: passed. node scripts/sps-surfaces-smoke.mjs: 16 screenshots passed including 04d-page-tree-dnd; SURFACES_SMOKE_DONE and persisted tree assertion passed.</x:v>
       </x:c>
       <x:c r="O24" s="9" t="str"/>
     </x:row>
@@ -4299,7 +4299,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94205b57b63c4b21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2585b5f05464122"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4427,7 +4427,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raff9ad353b18497f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a24a98ca615475e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5240,10 +5240,80 @@
         <x:v>15/15 behavior screenshots passed. Personal Health fresh/offline checks covered journal/protocol/document deletes via UI plus IPC readback, offline clinical digest render with 2 fallback articles, and no targeted health bootstrap console/page errors.</x:v>
       </x:c>
     </x:row>
+    <x:row r="58">
+      <x:c r="A58" t="str">
+        <x:v>2026-06-22</x:v>
+      </x:c>
+      <x:c r="B58" t="str">
+        <x:v>npm test -- --run src/renderer/src/screens/SpsAgent/store/workspace-dbcleanup.test.ts src/renderer/src/screens/SpsAgent/lib/tree.test.ts src/renderer/src/screens/SpsAgent/sidebar/TreeNode.test.tsx</x:v>
+      </x:c>
+      <x:c r="C58" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D58" t="str">
+        <x:v>3 files, 14 tests passed; covered nested subtree restore, legacy trash restore, permanent delete cleanup, shared DB-folder retention, treeMove, and TreeNode DnD zones.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" t="str">
+        <x:v>2026-06-22</x:v>
+      </x:c>
+      <x:c r="B59" t="str">
+        <x:v>npm test -- --run src/main/sps-vault.test.ts src/renderer/src/screens/SpsAgent/lib/vaultStore.test.ts</x:v>
+      </x:c>
+      <x:c r="C59" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D59" t="str">
+        <x:v>2 files, 40 tests passed for safe vault page and database-folder cleanup helpers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="str">
+        <x:v>2026-06-22</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>npm run typecheck</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D60" t="str">
+        <x:v>typecheck:node and typecheck:web completed successfully after adding TrashEntry.subtree.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
+        <x:v>2026-06-22</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>npm run build</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>typecheck, MCP bundles, and Electron/Vite production build completed successfully.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" t="str">
+        <x:v>2026-06-22</x:v>
+      </x:c>
+      <x:c r="B62" t="str">
+        <x:v>node scripts/sps-surfaces-smoke.mjs</x:v>
+      </x:c>
+      <x:c r="C62" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="D62" t="str">
+        <x:v>Escalated Electron launch passed 16/16 screenshots including 04d-page-tree-dnd; SURFACES_SMOKE_DONE and persisted workspace tree assertion passed.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b702bd8f58b4e18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9dd6dd32b574368"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>